<commit_message>
Moved around some connections and re-routed board.
</commit_message>
<xml_diff>
--- a/Project Outputs for Vehicle_Interface_Tester/BOM/Bill of Materials-Vehicle_Interface_Tester.xlsx
+++ b/Project Outputs for Vehicle_Interface_Tester/BOM/Bill of Materials-Vehicle_Interface_Tester.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_local\Vehicle_Interface_Tester_PCB\Project Outputs for Vehicle_Interface_Tester\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_Local\Vehicle_Interface_Tester_PCB\Project Outputs for Vehicle_Interface_Tester\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9ED0D0F1-F9FA-4BE2-A8AE-94F3C2EAC5BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F06F427E-3113-47B3-83FA-6FAB8D039CEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="5060" windowWidth="37450" windowHeight="11680" xr2:uid="{CE3CD6AD-04C6-4C04-BF63-6D96B3AD1D3D}"/>
+    <workbookView xWindow="2960" yWindow="2960" windowWidth="28800" windowHeight="15370" xr2:uid="{4BE05F64-0944-4A2B-B2F8-4D756A022366}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-Vehicle_Inter" sheetId="1" r:id="rId1"/>
@@ -1249,7 +1249,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C6A631F-4C32-451B-969A-2B90658A9F3F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E45152C-0D33-4954-8A04-F9839F1EE2A5}">
   <dimension ref="A1:F64"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>

<commit_message>
Made board 1mm smaller all around.
</commit_message>
<xml_diff>
--- a/Project Outputs for Vehicle_Interface_Tester/BOM/Bill of Materials-Vehicle_Interface_Tester.xlsx
+++ b/Project Outputs for Vehicle_Interface_Tester/BOM/Bill of Materials-Vehicle_Interface_Tester.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_Local\Vehicle_Interface_Tester_PCB\Project Outputs for Vehicle_Interface_Tester\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_local\Vehicle_Interface_Tester_PCB\Project Outputs for Vehicle_Interface_Tester\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F06F427E-3113-47B3-83FA-6FAB8D039CEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{714EBCB0-82BD-4AAE-B700-1BF6938AEF98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2960" yWindow="2960" windowWidth="28800" windowHeight="15370" xr2:uid="{4BE05F64-0944-4A2B-B2F8-4D756A022366}"/>
+    <workbookView xWindow="0" yWindow="5060" windowWidth="37450" windowHeight="11680" xr2:uid="{27673614-06F9-46B9-BBEB-8F2196639A43}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-Vehicle_Inter" sheetId="1" r:id="rId1"/>
@@ -1249,7 +1249,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E45152C-0D33-4954-8A04-F9839F1EE2A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3698F2BB-F6DD-40DC-BB01-F731B829B4BF}">
   <dimension ref="A1:F64"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>

<commit_message>
Ordered from JLC PCB 10/28/2026
</commit_message>
<xml_diff>
--- a/Project Outputs for Vehicle_Interface_Tester/BOM/Bill of Materials-Vehicle_Interface_Tester.xlsx
+++ b/Project Outputs for Vehicle_Interface_Tester/BOM/Bill of Materials-Vehicle_Interface_Tester.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_local\Vehicle_Interface_Tester_PCB\Project Outputs for Vehicle_Interface_Tester\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_Local\Vehicle_Interface_Tester_PCB\Project Outputs for Vehicle_Interface_Tester\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{714EBCB0-82BD-4AAE-B700-1BF6938AEF98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8AD4937E-D0D4-4468-8748-D46FD412F2B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="5060" windowWidth="37450" windowHeight="11680" xr2:uid="{27673614-06F9-46B9-BBEB-8F2196639A43}"/>
+    <workbookView xWindow="2960" yWindow="2960" windowWidth="28800" windowHeight="15370" xr2:uid="{32E4B132-EBE2-43AC-B5CD-D9D365096989}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-Vehicle_Inter" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="279">
   <si>
     <t>Designator</t>
   </si>
@@ -222,7 +222,7 @@
     <t>22uF</t>
   </si>
   <si>
-    <t>D1, D8, D9</t>
+    <t>D1, D9</t>
   </si>
   <si>
     <t>Schottky Diode, 5A, 30V, SOD-128</t>
@@ -666,94 +666,85 @@
     <t>10M</t>
   </si>
   <si>
-    <t>R11, R12</t>
-  </si>
-  <si>
-    <t>2K ohm, ±1%, 0603 (1608)</t>
-  </si>
-  <si>
-    <t>C22975</t>
+    <t>R13, R14, R15</t>
+  </si>
+  <si>
+    <t>4.7K ohm, Resistor, ±1%, 0402 (1005)</t>
+  </si>
+  <si>
+    <t>C25900</t>
+  </si>
+  <si>
+    <t>4.7K</t>
+  </si>
+  <si>
+    <t>R17</t>
+  </si>
+  <si>
+    <t>2.2K ohm, Resistor, ±1%, 1/4W, 1206 (3216)</t>
+  </si>
+  <si>
+    <t>C17948</t>
+  </si>
+  <si>
+    <t>2.2K</t>
+  </si>
+  <si>
+    <t>R18</t>
+  </si>
+  <si>
+    <t>1K ohm, Resistor, ±1%, 0402 (1005)</t>
+  </si>
+  <si>
+    <t>C11702</t>
+  </si>
+  <si>
+    <t>1K</t>
+  </si>
+  <si>
+    <t>R20</t>
+  </si>
+  <si>
+    <t>100K ohm, Resistor, ±1%, 0402 (1005)</t>
+  </si>
+  <si>
+    <t>C25741</t>
+  </si>
+  <si>
+    <t>R22</t>
+  </si>
+  <si>
+    <t>13K ohm, Resistor, ±1%, 0402 (1005)</t>
+  </si>
+  <si>
+    <t>C25754</t>
+  </si>
+  <si>
+    <t>13K</t>
+  </si>
+  <si>
+    <t>R23</t>
+  </si>
+  <si>
+    <t>21K ohm, Resistor, ±1%, 0402 (1005)</t>
+  </si>
+  <si>
+    <t>C25766</t>
+  </si>
+  <si>
+    <t>21K</t>
+  </si>
+  <si>
+    <t>R24</t>
+  </si>
+  <si>
+    <t>2K ohm, Resistor, ±1%, 0402 (1005)</t>
+  </si>
+  <si>
+    <t>C4109</t>
   </si>
   <si>
     <t>2K</t>
-  </si>
-  <si>
-    <t>R13, R14, R15</t>
-  </si>
-  <si>
-    <t>4.7K ohm, Resistor, ±1%, 0402 (1005)</t>
-  </si>
-  <si>
-    <t>C25900</t>
-  </si>
-  <si>
-    <t>4.7K</t>
-  </si>
-  <si>
-    <t>R17</t>
-  </si>
-  <si>
-    <t>2.2K ohm, Resistor, ±1%, 1/4W, 1206 (3216)</t>
-  </si>
-  <si>
-    <t>C17948</t>
-  </si>
-  <si>
-    <t>2.2K</t>
-  </si>
-  <si>
-    <t>R18</t>
-  </si>
-  <si>
-    <t>1K ohm, Resistor, ±1%, 0402 (1005)</t>
-  </si>
-  <si>
-    <t>C11702</t>
-  </si>
-  <si>
-    <t>1K</t>
-  </si>
-  <si>
-    <t>R20</t>
-  </si>
-  <si>
-    <t>100K ohm, Resistor, ±1%, 0402 (1005)</t>
-  </si>
-  <si>
-    <t>C25741</t>
-  </si>
-  <si>
-    <t>R22</t>
-  </si>
-  <si>
-    <t>13K ohm, Resistor, ±1%, 0402 (1005)</t>
-  </si>
-  <si>
-    <t>C25754</t>
-  </si>
-  <si>
-    <t>13K</t>
-  </si>
-  <si>
-    <t>R23</t>
-  </si>
-  <si>
-    <t>21K ohm, Resistor, ±1%, 0402 (1005)</t>
-  </si>
-  <si>
-    <t>C25766</t>
-  </si>
-  <si>
-    <t>21K</t>
-  </si>
-  <si>
-    <t>R24</t>
-  </si>
-  <si>
-    <t>2K ohm, Resistor, ±1%, 0402 (1005)</t>
-  </si>
-  <si>
-    <t>C4109</t>
   </si>
   <si>
     <t>R25</t>
@@ -1249,8 +1240,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3698F2BB-F6DD-40DC-BB01-F731B829B4BF}">
-  <dimension ref="A1:F64"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5DC0D7E-C4ED-47C1-8CA3-69980585A979}">
+  <dimension ref="A1:F63"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="18.81640625" customWidth="1"/>
@@ -1566,7 +1557,7 @@
         <v>65</v>
       </c>
       <c r="C16" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>66</v>
@@ -2206,13 +2197,13 @@
         <v>213</v>
       </c>
       <c r="C48" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>214</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>215</v>
@@ -2226,13 +2217,13 @@
         <v>217</v>
       </c>
       <c r="C49" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>218</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>219</v>
@@ -2252,7 +2243,7 @@
         <v>222</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>223</v>
@@ -2275,27 +2266,27 @@
         <v>24</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>227</v>
+        <v>203</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="B52" s="2" t="s">
+      <c r="C52" s="1">
+        <v>1</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>229</v>
-      </c>
-      <c r="C52" s="1">
-        <v>1</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>230</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>203</v>
+        <v>230</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
@@ -2355,187 +2346,167 @@
         <v>24</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>215</v>
+        <v>242</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C56" s="1">
         <v>1</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C57" s="1">
         <v>1</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C58" s="1">
         <v>1</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C59" s="1">
         <v>1</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>24</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C60" s="1">
         <v>1</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>24</v>
+        <v>262</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C61" s="1">
         <v>1</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C62" s="1">
         <v>1</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C63" s="1">
         <v>1</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A64" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="B64" s="2" t="s">
         <v>278</v>
-      </c>
-      <c r="C64" s="1">
-        <v>1</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>280</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>